<commit_message>
João: facto estilizado 7 (persistência do volume)
</commit_message>
<xml_diff>
--- a/data/processed/calibracao_log.xlsx
+++ b/data/processed/calibracao_log.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:AA2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -455,6 +455,7 @@
     <col width="14" customWidth="1" min="24" max="24"/>
     <col width="14" customWidth="1" min="25" max="25"/>
     <col width="80" customWidth="1" min="26" max="26"/>
+    <col width="80" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1" ht="60" customHeight="1">
@@ -580,10 +581,15 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
+          <t>Autocorr volume (alvo &gt;0)</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
           <t>Factos que batem</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Diagnóstico e decisão</t>
         </is>
@@ -668,14 +674,17 @@
       <c r="X2" t="n">
         <v>0.2043</v>
       </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>1 / 6</t>
-        </is>
-      </c>
-      <c r="Z2" s="2" t="inlineStr">
-        <is>
-          <t>Mercado 5× calmo demais. A volatilidade vem quase só das notícias (1 a cada 5 dias, ±1% → 0.44%/dia em teoria, 0.42% no modelo) e os fundamentalistas prendem o preço ao valor fundamental (autocorrelação −0.14). A curtose média de 9.6 vem de 3 corridas com reservas; a mediana é 0.2. Próxima ronda: newsRate 0.0004 → 0.002 e notícia ±1% → ±2% (teoria: vol 2.0%, curtose 2.9, 13.7% de dias &gt;3%).</t>
+      <c r="Y2" t="n">
+        <v>0.0401</v>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>2 / 7</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>Mercado 5× calmo demais. A volatilidade vem quase só das notícias (1 a cada 5 dias, ±1% → 0.44%/dia em teoria, 0.42% no modelo) e os fundamentalistas prendem o preço ao valor fundamental (autocorrelação −0.14). A curtose média de 9.6 vem de 3 corridas com reservas; a mediana é 0.2. Próxima ronda: newsRate 0.0004 → 0.002 e notícia ±1% → ±2% (teoria: vol 2.0%, curtose 2.9, 13.7% de dias &gt;3%). Facto 7 (persistência do volume) acrescentado a 31/10, antes da ronda 1: na ronda 0 deu 0.040 (mediana 0.021), bate por pouco.</t>
         </is>
       </c>
     </row>

</xml_diff>